<commit_message>
docs: publish completed physical Y and early identity Z evidence
</commit_message>
<xml_diff>
--- a/deliverables/verified_20260910/model_y/selected/official-report.xlsx
+++ b/deliverables/verified_20260910/model_y/selected/official-report.xlsx
@@ -603,14 +603,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Источник: /root/projects/TimesOil/results/audit-20260909/timesfm-monthly-y-v5-20260909/opm/opm-full-replay-5b12ea50006b3bb1c213439c/.chdd-ndu6mdwn/input.csv  |  Период: 2014–2015  |  Версия ядра: 7.0.2-negative-row-filter</t>
+          <t>Источник: /root/projects/TimesOil/results/audit-20260909/physical-only-monthly-y-20260910/opm/opm-full-replay-4769989869d96c2be60ba2ff/.chdd-d60pcmug/input.csv  |  Период: 2014–2015  |  Версия ядра: 7.0.2-negative-row-filter</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Итоговый ЧДД: 1 597.088 млн руб.   |   ИДДз: 1.199   |   Остановки/запуски: 1 событий   |   Переводы под закачку: 0</t>
+          <t>Итоговый ЧДД: 1 596.778 млн руб.   |   ИДДз: 1.199   |   Остановки/запуски: 1 событий   |   Переводы под закачку: 0</t>
         </is>
       </c>
     </row>
@@ -661,10 +661,10 @@
         </is>
       </c>
       <c r="D7" s="9" t="n">
-        <v>7576.599470567206</v>
+        <v>7576.691741203713</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>9261.554694505547</v>
+        <v>9261.613252528867</v>
       </c>
     </row>
     <row r="8">
@@ -684,10 +684,10 @@
         </is>
       </c>
       <c r="D8" s="13" t="n">
-        <v>1398.719874915584</v>
+        <v>1398.69750456384</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>1541.28249316288</v>
+        <v>1541.264334811968</v>
       </c>
     </row>
     <row r="9">
@@ -707,10 +707,10 @@
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>7880.7506875</v>
+        <v>7880.80378125</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>9539.86634375</v>
+        <v>9539.92271875</v>
       </c>
     </row>
     <row r="10">
@@ -730,10 +730,10 @@
         </is>
       </c>
       <c r="D10" s="13" t="n">
-        <v>2022.328726294266</v>
+        <v>2022.420996930773</v>
       </c>
       <c r="E10" s="13" t="n">
-        <v>1684.955223938341</v>
+        <v>1684.921511325153</v>
       </c>
     </row>
     <row r="11">
@@ -753,10 +753,10 @@
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>214.296527252288</v>
+        <v>214.274156900544</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>142.5626182472959</v>
+        <v>142.566830248128</v>
       </c>
     </row>
     <row r="12">
@@ -776,10 +776,10 @@
         </is>
       </c>
       <c r="D12" s="13" t="n">
-        <v>1991.56384375</v>
+        <v>1991.6169375</v>
       </c>
       <c r="E12" s="13" t="n">
-        <v>1659.11565625</v>
+        <v>1659.1189375</v>
       </c>
     </row>
     <row r="13">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D13" s="9" t="n">
-        <v>48</v>
+        <v>48.25</v>
       </c>
       <c r="E13" s="9" t="n">
         <v>48</v>
@@ -822,7 +822,7 @@
         </is>
       </c>
       <c r="D14" s="14" t="n">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="E14" s="14" t="n">
         <v>528</v>
@@ -845,10 +845,10 @@
         </is>
       </c>
       <c r="D15" s="9" t="n">
-        <v>174.9273416276042</v>
+        <v>173.5799824315245</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>158.5352632954545</v>
+        <v>158.5321977357955</v>
       </c>
     </row>
     <row r="16">
@@ -868,10 +868,10 @@
         </is>
       </c>
       <c r="D16" s="13" t="n">
-        <v>18.36202834483333</v>
+        <v>18.21779288326615</v>
       </c>
       <c r="E16" s="13" t="n">
-        <v>13.34460127</v>
+        <v>13.34499574672727</v>
       </c>
     </row>
     <row r="17">
@@ -891,10 +891,10 @@
         </is>
       </c>
       <c r="D17" s="9" t="n">
-        <v>341.0416960416667</v>
+        <v>341.0506933958333</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>310.4406599545455</v>
+        <v>310.4412742897727</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
@@ -1648,10 +1648,10 @@
         </is>
       </c>
       <c r="D52" s="13" t="n">
-        <v>6000.302763064065</v>
+        <v>5999.676393215232</v>
       </c>
       <c r="E52" s="13" t="n">
-        <v>3991.753310924286</v>
+        <v>3991.871246947585</v>
       </c>
     </row>
     <row r="53">
@@ -1671,10 +1671,10 @@
         </is>
       </c>
       <c r="D53" s="9" t="n">
-        <v>8.571861090091522</v>
+        <v>8.570966276021759</v>
       </c>
       <c r="E53" s="9" t="n">
-        <v>5.702504729891837</v>
+        <v>5.702673209925121</v>
       </c>
     </row>
     <row r="54">
@@ -1694,10 +1694,10 @@
         </is>
       </c>
       <c r="D54" s="13" t="n">
-        <v>202.2328726294266</v>
+        <v>202.2420996930773</v>
       </c>
       <c r="E54" s="13" t="n">
-        <v>168.4955223938341</v>
+        <v>168.4921511325153</v>
       </c>
     </row>
     <row r="55">
@@ -1717,10 +1717,10 @@
         </is>
       </c>
       <c r="D55" s="9" t="n">
-        <v>59.7469153125</v>
+        <v>59.748508125</v>
       </c>
       <c r="E55" s="9" t="n">
-        <v>49.7734696875</v>
+        <v>49.773568125</v>
       </c>
     </row>
     <row r="56">
@@ -1740,7 +1740,7 @@
         </is>
       </c>
       <c r="D56" s="13" t="n">
-        <v>48</v>
+        <v>48.25</v>
       </c>
       <c r="E56" s="13" t="n">
         <v>44</v>
@@ -1786,10 +1786,10 @@
         </is>
       </c>
       <c r="D58" s="13" t="n">
-        <v>373.5516490320181</v>
+        <v>373.8115740940991</v>
       </c>
       <c r="E58" s="13" t="n">
-        <v>267.9714968112259</v>
+        <v>267.9683924674405</v>
       </c>
     </row>
     <row r="59">
@@ -1855,10 +1855,10 @@
         </is>
       </c>
       <c r="D61" s="9" t="n">
-        <v>4200.211934144846</v>
+        <v>4199.773475250662</v>
       </c>
       <c r="E61" s="9" t="n">
-        <v>2794.227317647</v>
+        <v>2794.309872863309</v>
       </c>
     </row>
     <row r="62">
@@ -1878,10 +1878,10 @@
         </is>
       </c>
       <c r="D62" s="13" t="n">
-        <v>1426.539179887201</v>
+        <v>1426.091343870471</v>
       </c>
       <c r="E62" s="13" t="n">
-        <v>929.55449646606</v>
+        <v>929.5929816168349</v>
       </c>
     </row>
     <row r="63">
@@ -1901,10 +1901,10 @@
         </is>
       </c>
       <c r="D63" s="9" t="n">
-        <v>356.6347949718004</v>
+        <v>356.5228359676177</v>
       </c>
       <c r="E63" s="9" t="n">
-        <v>232.388624116515</v>
+        <v>232.3982454042087</v>
       </c>
     </row>
     <row r="64">
@@ -1924,10 +1924,10 @@
         </is>
       </c>
       <c r="D64" s="13" t="n">
-        <v>1426.539179887201</v>
+        <v>1426.091343870471</v>
       </c>
       <c r="E64" s="13" t="n">
-        <v>929.55449646606</v>
+        <v>929.5929816168349</v>
       </c>
     </row>
     <row r="65">
@@ -1947,10 +1947,10 @@
         </is>
       </c>
       <c r="D65" s="9" t="n">
-        <v>963.3004149154011</v>
+        <v>962.964537902853</v>
       </c>
       <c r="E65" s="9" t="n">
-        <v>697.165872349545</v>
+        <v>697.1947362126261</v>
       </c>
     </row>
     <row r="66">
@@ -1993,10 +1993,10 @@
         </is>
       </c>
       <c r="D67" s="9" t="n">
-        <v>963.3004149154011</v>
+        <v>962.964537902853</v>
       </c>
       <c r="E67" s="9" t="n">
-        <v>633.7871566814044</v>
+        <v>633.8133965569328</v>
       </c>
     </row>
     <row r="68">
@@ -2016,10 +2016,10 @@
         </is>
       </c>
       <c r="D68" s="13" t="n">
-        <v>963.3004149154011</v>
+        <v>962.964537902853</v>
       </c>
       <c r="E68" s="13" t="n">
-        <v>1597.087571596805</v>
+        <v>1596.777934459786</v>
       </c>
     </row>
     <row r="69">
@@ -2039,10 +2039,10 @@
         </is>
       </c>
       <c r="D69" s="9" t="n">
-        <v>6000.302763064065</v>
+        <v>5999.676393215232</v>
       </c>
       <c r="E69" s="9" t="n">
-        <v>3628.866646294805</v>
+        <v>3628.973860861441</v>
       </c>
     </row>
     <row r="70">
@@ -2062,10 +2062,10 @@
         </is>
       </c>
       <c r="D70" s="13" t="n">
-        <v>5037.002348148664</v>
+        <v>5036.711855312378</v>
       </c>
       <c r="E70" s="13" t="n">
-        <v>2995.079489613401</v>
+        <v>2995.160464304508</v>
       </c>
     </row>
     <row r="71">
@@ -2085,10 +2085,10 @@
         </is>
       </c>
       <c r="D71" s="22" t="n">
-        <v>1.191244781783646</v>
+        <v>1.191189126073826</v>
       </c>
       <c r="E71" s="22" t="n">
-        <v>1.198838558154158</v>
+        <v>1.198805193972002</v>
       </c>
     </row>
     <row r="72">
@@ -2114,7 +2114,7 @@
         <v>-1.4210854715202e-14</v>
       </c>
       <c r="E73" s="24" t="n">
-        <v>2.842170943040401e-14</v>
+        <v>-2.842170943040401e-14</v>
       </c>
     </row>
     <row r="74">

</xml_diff>